<commit_message>
upload pack 009 and 010, Compact/expandable Notes and Riffs fields; reorder detail view sections
</commit_message>
<xml_diff>
--- a/content/packs/pack-010.xlsx
+++ b/content/packs/pack-010.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH2"/>
+  <dimension ref="A1:AH4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -723,6 +723,290 @@
         </is>
       </c>
       <c r="AH2" t="inlineStr">
+        <is>
+          <t>modern</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>treacle-no1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Treacle No.1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>old-fashioned</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Old Fashioned</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>core-old-fashioned</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Core Old Fashioned</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Rum</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>rocks-old-fashioned</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Rocks/Old Fashioned</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>On the Rocks</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Nightcap</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Fall</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Boozy,Rich,Bitter,Herbal/Botanical</t>
+        </is>
+      </c>
+      <c r="O3" t="n">
+        <v>7</v>
+      </c>
+      <c r="P3" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>3</v>
+      </c>
+      <c r="S3" t="n">
+        <v>2</v>
+      </c>
+      <c r="T3" t="n">
+        <v>2</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" t="n">
+        <v>1</v>
+      </c>
+      <c r="W3" t="n">
+        <v>7</v>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>pack-010</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>draft_needs_review</t>
+        </is>
+      </c>
+      <c r="AA3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>Treacle</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>https://www.diffordsguide.com/cocktails/recipe/1983/treacle-no1</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>Dick Bradsell</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>Independent / London bar scene</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>modern</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>twinkle</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Twinkle</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>spritz-aperitivo</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Spritz &amp; Aperitivo</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>royale</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Royale</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Vodka</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>coupe</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Coupe</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Party</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Spring</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Light/Refreshing,Sparkling,Floral,Elegant</t>
+        </is>
+      </c>
+      <c r="O4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" t="n">
+        <v>2</v>
+      </c>
+      <c r="T4" t="n">
+        <v>3</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" t="n">
+        <v>1</v>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>pack-010</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>draft_needs_review</t>
+        </is>
+      </c>
+      <c r="AA4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>https://www.diffordsguide.com/cocktails/recipe/2007/twinkle</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>Tony Conigliaro</t>
+        </is>
+      </c>
+      <c r="AF4" t="n">
+        <v>2002</v>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>The Lonsdale, London</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
         <is>
           <t>modern</t>
         </is>
@@ -739,7 +1023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -813,6 +1097,80 @@
       <c r="G2" t="inlineStr">
         <is>
           <t>The Monella Sour is a window into what contemporary Italian cocktail culture looks like outside of Milan and Rome — a small bar on a small island, run by someone with serious international pedigree, making something genuinely original. It also demonstrates how well cinnamon functions as the primary spice modifier in a citrus sour: most cinnamon drinks use it as an accent; here it's the point.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>treacle-no1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Dick Bradsell heard a story about the decline of the British apple farming industry — how the orchards were disappearing, how the juice that remained was the cheap concentrated stuff, pressed into cartons. He filed it away. He already loved Myers's Dark Rum, which he thought was underrated and underused. At some point in 1990s London, the two things came together over ice in a rocks glass, and the Treacle was born. Bradsell was the godfather of modern British bartending: the Bramble, the Espresso Martini, the Russian Spring Punch all came from his hands. He worked at Zanzibar, The Player, Atlantic Bar &amp; Grill, and Match — bars that defined London cocktail culture in the era before craft became a word anyone used. His protégés are now the senior figures of the international bar world. Vincenzo Errico, who trained under him, later created the Red Hook at Milk &amp; Honey and eventually opened L'ArteFatto on Ischia. Bradsell died in 2016. The Treacle, written down in his own words in Dicktales (2022), is one of the cleaner windows into how he thought: simple materials, a strong opinion about which version of apple juice was correct, and a technique that made the building of the drink part of its character.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Bradsell was emphatic about the apple juice: clear from concentrate — the cheap supermarket carton — not pressed/cloudy. The clear juice produces the treacly, caramelized quality the drink is named for; pressed juice pulls it in a fresher, fruitier direction that he considered a different drink. Simon Difford personally prefers pressed juice (reducing sugar accordingly), but acknowledges this departs from Bradsell's intent. The two-pour technique is canonical: split the rum in half, build with ice and stir between pours, then float the apple juice at the end rather than stirring it in. Myers's is the named rum; any funky Jamaican pot-still rum (Smith &amp; Cross, Appleton Estate 12, Hamilton Pot Still Black) works well. Lighter aged rums fall short — the funk is load-bearing. Bradsell's original spec from Dicktales (2022): "Into an old fashioned glass — 1 barspoon cane sugar syrup, 2 dashes of Angostura, stir with 1 cube of ice, add 25mls Myers rum, 1 cube ice and stir, and two cubes ice stir, 25mls Myers and stir, 1 ice cube stir, 20mls concentrated apple juice (the cheap clear stuff), garnish a lemon twist (or two)."</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Split the rum between Myers's and a lighter Spanish-style aged rum for more balance with less funk. Use a barspoon of demerara syrup instead of cane sugar for a deeper, more bitter-molasses quality. A Peychaud's dash alongside the Angostura adds a faint anise note and brightens the colour.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Deep molasses and dark fruit on the nose — rum-forward with a hint of toffee apple. On the palate: rich, warming, slightly bitter from the bitters, with the apple juice arriving late as a bright, almost cidery lift. Long finish, dry and spiced.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Difford's Guide named the Treacle No.1 its cocktail of the day on January 15th — the anniversary of the 1919 Boston Molasses Disaster, when a storage tank burst and flooded Boston's North End with 2.3 million gallons of molasses at 35 mph. The connection is apt. The drink tastes exactly like that sounds.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>The Treacle is a Rum Old Fashioned, but it matters because of who made it and what it says about his thinking. Bradsell's instinct was always to find the unexpected pairing — espresso and vodka, rum and industrial apple juice — and trust it rather than finesse it. The drink is also a study in technique: the build-in-glass method, the split pour, the late float aren't affectations but ways of controlling dilution and layering flavor. It's a teaching drink disguised as a simple one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>twinkle</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Tony Conigliaro made the Twinkle at The Lonsdale in London in 2002 — five years before St-Germain existed. That timing matters: the drink was built around elderflower cordial, the humble British pantry staple, not the French liqueur that would later become synonymous with the flavor. When St-Germain arrived in 2007 and swept through the world's cocktail bars, the Twinkle migrated with it, the cordial replaced by the liqueur almost everywhere the drink was made. The original is the better argument for cordial. Conigliaro trained under Dick Bradsell — the man who defined British bartending in the 1980s and '90s — and went on to become the most scientifically rigorous bartender of his generation. He ran 69 Colebrooke Row, a bar in Islington that operated more like a research kitchen than a cocktail lounge, and his book The Cocktail Lab won the James Beard Award for best beverage book in 2014. The Twinkle is the other side of that coin: before the centrifuges and the fat-washes, there was this — a drink so clean and light it barely seems like it's happening, right up until it isn't.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>The original spec (2002) uses elderflower cordial and prosecco. The now-common adaptation substitutes St-Germain elderflower liqueur and champagne — the liqueur reads richer and more floral, the cordial drier and more delicate. Use less cordial than you think (0.5oz is the ceiling; 0.33oz is worth trying). The vodka should be clean and neutral — this is not the place for character. Do not stir in the sparkling wine; top gently and let it integrate.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Substitute gin for vodka for a more botanical version — a London dry works best, nothing too floral. Use Lillet Blanc in place of half the vodka for a wine-forward, lower-ABV take. A few drops of citrus bitters before topping add a gentle counterpoint to the elderflower sweetness.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Pale gold, fine bubbles. Elderflower on the nose — delicate, just-picked, with a clean lemon lift. Light-bodied on the palate, dry, with the vodka providing structure behind the floral softness. Champagne carries it out long and bright.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>The Twinkle predates St-Germain by five years. Every bar that makes it with elderflower liqueur today is unknowingly using an adaptation. The original was built around cordial — and it was better that way.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>The Twinkle is a study in restraint from a bartender better known for complexity. Three ingredients, perfectly balanced, requiring almost nothing technically. It also marks a specific moment in cocktail history: the early 2000s London bar scene that Bradsell's generation built, just before St-Germain, the Aperol Spritz, and the broader craft wave reshaped what people were drinking. This drink is from the quiet moment just before.</t>
         </is>
       </c>
     </row>
@@ -827,7 +1185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -851,6 +1209,30 @@
       <c r="B2" t="inlineStr">
         <is>
           <t>[{"name":"Vodka","amount":"1.5","unit":"oz"},{"name":"Orange juice","amount":"1","unit":"oz"},{"name":"Cinnamon syrup, Liber &amp; Co.","amount":"0.5","unit":"oz"},{"name":"Lime juice","amount":"0.5","unit":"oz"}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>treacle-no1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>[{"name":"Aged Jamaican rum, Myers's","amount":"1","unit":"oz"},{"name":"Rich simple syrup, 2:1","amount":"0.25","unit":"oz"},{"name":"Angostura bitters","amount":"2","unit":"dash"},{"name":"Aged Jamaican rum, Myers's","amount":"1","unit":"oz"},{"name":"Clear apple juice","amount":"0.75","unit":"oz"}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>twinkle</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>[{"name":"Vodka","amount":"2","unit":"oz"},{"name":"Elderflower cordial","amount":"0.5","unit":"oz"},{"name":"Prosecco or brut champagne","amount":"2","unit":"oz"}]</t>
         </is>
       </c>
     </row>
@@ -865,7 +1247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -892,6 +1274,30 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>treacle-no1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Pour first ounce of rum, sugar syrup, and bitters into a rocks glass. Add two ice cubes and stir. Add second ounce of rum, two more ice cubes, and stir again. Fill glass with ice and stir once more. Float the apple juice over the top — do not stir in. Express a lemon twist over the glass and use as garnish.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>twinkle</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Add vodka and elderflower cordial to a shaker with ice. Shake until well chilled. Fine-strain into a chilled coupe. Top gently with prosecco or brut champagne. Express a lemon twist over the glass and use as garnish.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>